<commit_message>
new runs of codes
</commit_message>
<xml_diff>
--- a/code/resultados/NWJSSP_OADG_EPR(VND).xlsx
+++ b/code/resultados/NWJSSP_OADG_EPR(VND).xlsx
@@ -12,6 +12,9 @@
     <sheet name="ft10" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="ft10r" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="ft20" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ft20r" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="tai_j10_m10_1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="tai_j10_m10_1r" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -619,6 +622,228 @@
       <c r="B1" t="n">
         <v>246309</v>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B2" t="n">
+        <v>152</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1050</v>
+      </c>
+      <c r="D2" t="n">
+        <v>598</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>186</v>
+      </c>
+      <c r="G2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H2" t="n">
+        <v>118</v>
+      </c>
+      <c r="I2" t="n">
+        <v>263</v>
+      </c>
+      <c r="J2" t="n">
+        <v>849</v>
+      </c>
+      <c r="K2" t="n">
+        <v>359</v>
+      </c>
+      <c r="L2" t="n">
+        <v>844</v>
+      </c>
+      <c r="M2" t="n">
+        <v>570</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1400</v>
+      </c>
+      <c r="O2" t="n">
+        <v>1215</v>
+      </c>
+      <c r="P2" t="n">
+        <v>769</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>490</v>
+      </c>
+      <c r="R2" t="n">
+        <v>1247</v>
+      </c>
+      <c r="S2" t="n">
+        <v>976</v>
+      </c>
+      <c r="T2" t="n">
+        <v>557</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>17290</v>
+      </c>
+      <c r="B1" t="n">
+        <v>284395</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1162</v>
+      </c>
+      <c r="C2" t="n">
+        <v>662</v>
+      </c>
+      <c r="D2" t="n">
+        <v>362</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>882</v>
+      </c>
+      <c r="G2" t="n">
+        <v>299</v>
+      </c>
+      <c r="H2" t="n">
+        <v>199</v>
+      </c>
+      <c r="I2" t="n">
+        <v>863</v>
+      </c>
+      <c r="J2" t="n">
+        <v>535</v>
+      </c>
+      <c r="K2" t="n">
+        <v>81</v>
+      </c>
+      <c r="L2" t="n">
+        <v>94</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1345</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1151</v>
+      </c>
+      <c r="O2" t="n">
+        <v>830</v>
+      </c>
+      <c r="P2" t="n">
+        <v>533</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>406</v>
+      </c>
+      <c r="R2" t="n">
+        <v>1476</v>
+      </c>
+      <c r="S2" t="n">
+        <v>1031</v>
+      </c>
+      <c r="T2" t="n">
+        <v>263</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>94122</v>
+      </c>
+      <c r="B1" t="n">
+        <v>44909</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="n">
+        <v>118</v>
+      </c>
+      <c r="C2" t="n">
+        <v>4829</v>
+      </c>
+      <c r="D2" t="n">
+        <v>7278</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5204</v>
+      </c>
+      <c r="F2" t="n">
+        <v>8183</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3140</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>8786</v>
+      </c>
+      <c r="J2" t="n">
+        <v>3829</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>94122</v>
+      </c>
+      <c r="B1" t="n">
+        <v>37016</v>
+      </c>
       <c r="C1" t="inlineStr"/>
       <c r="D1" t="inlineStr"/>
       <c r="E1" t="inlineStr"/>
@@ -627,77 +852,37 @@
       <c r="H1" t="inlineStr"/>
       <c r="I1" t="inlineStr"/>
       <c r="J1" t="inlineStr"/>
-      <c r="K1" t="inlineStr"/>
-      <c r="L1" t="inlineStr"/>
-      <c r="M1" t="inlineStr"/>
-      <c r="N1" t="inlineStr"/>
-      <c r="O1" t="inlineStr"/>
-      <c r="P1" t="inlineStr"/>
-      <c r="Q1" t="inlineStr"/>
-      <c r="R1" t="inlineStr"/>
-      <c r="S1" t="inlineStr"/>
-      <c r="T1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>152</v>
+        <v>118</v>
       </c>
       <c r="C2" t="n">
-        <v>1050</v>
+        <v>4829</v>
       </c>
       <c r="D2" t="n">
-        <v>598</v>
+        <v>7278</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>5204</v>
       </c>
       <c r="F2" t="n">
-        <v>186</v>
+        <v>8183</v>
       </c>
       <c r="G2" t="n">
-        <v>45</v>
+        <v>3140</v>
       </c>
       <c r="H2" t="n">
-        <v>118</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>263</v>
+        <v>8786</v>
       </c>
       <c r="J2" t="n">
-        <v>849</v>
-      </c>
-      <c r="K2" t="n">
-        <v>359</v>
-      </c>
-      <c r="L2" t="n">
-        <v>844</v>
-      </c>
-      <c r="M2" t="n">
-        <v>570</v>
-      </c>
-      <c r="N2" t="n">
-        <v>1400</v>
-      </c>
-      <c r="O2" t="n">
-        <v>1215</v>
-      </c>
-      <c r="P2" t="n">
-        <v>769</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>490</v>
-      </c>
-      <c r="R2" t="n">
-        <v>1247</v>
-      </c>
-      <c r="S2" t="n">
-        <v>976</v>
-      </c>
-      <c r="T2" t="n">
-        <v>557</v>
+        <v>3829</v>
       </c>
     </row>
   </sheetData>

</xml_diff>